<commit_message>
Update to the latest
</commit_message>
<xml_diff>
--- a/Data of test system 2.xlsx
+++ b/Data of test system 2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\workspace\GithubClone\supplementary files of collaborative operation of IES and TN\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\workspace\GithubClone\collaborative operation of IES and TN data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4909E238-98BE-42E0-B521-F8F07989D0D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{435F9A70-C628-4890-8003-23C90A1E678D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-107" yWindow="-107" windowWidth="41480" windowHeight="22717" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-104" yWindow="-104" windowWidth="39989" windowHeight="21859" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Energy demand" sheetId="1" r:id="rId1"/>
@@ -751,79 +751,79 @@
         <v>52</v>
       </c>
       <c r="C2" s="1">
-        <v>222.9999</v>
+        <v>2.7874987500000001</v>
       </c>
       <c r="D2" s="1">
-        <v>222.55629999999999</v>
+        <v>2.78195375</v>
       </c>
       <c r="E2" s="1">
-        <v>222.36775</v>
+        <v>2.7795968750000002</v>
       </c>
       <c r="F2" s="1">
-        <v>222.88145</v>
+        <v>2.786018125</v>
       </c>
       <c r="G2" s="1">
-        <v>222.59025</v>
+        <v>2.7823781250000001</v>
       </c>
       <c r="H2" s="1">
-        <v>225.03559999999999</v>
+        <v>2.812945</v>
       </c>
       <c r="I2" s="1">
-        <v>229.9829</v>
+        <v>2.8747862500000001</v>
       </c>
       <c r="J2" s="1">
-        <v>231.88075000000001</v>
+        <v>2.8985093750000002</v>
       </c>
       <c r="K2" s="1">
-        <v>237.11949999999999</v>
+        <v>2.9639937499999998</v>
       </c>
       <c r="L2" s="1">
-        <v>235.3425</v>
+        <v>2.94178125</v>
       </c>
       <c r="M2" s="1">
-        <v>233.86369999999999</v>
+        <v>2.9232962499999999</v>
       </c>
       <c r="N2" s="1">
-        <v>232.27379999999999</v>
+        <v>2.9034225</v>
       </c>
       <c r="Q2" t="s">
         <v>73</v>
       </c>
       <c r="R2" s="1">
-        <v>10</v>
+        <v>0.2</v>
       </c>
       <c r="S2" s="1">
-        <v>9.99</v>
+        <v>0.19980000000000001</v>
       </c>
       <c r="T2" s="1">
-        <v>9.93</v>
+        <v>0.1986</v>
       </c>
       <c r="U2" s="1">
-        <v>9.9700000000000006</v>
+        <v>0.19940000000000002</v>
       </c>
       <c r="V2" s="1">
-        <v>10.01</v>
+        <v>0.20019999999999999</v>
       </c>
       <c r="W2" s="1">
-        <v>10.28</v>
+        <v>0.20559999999999998</v>
       </c>
       <c r="X2" s="1">
-        <v>11.46</v>
+        <v>0.22920000000000001</v>
       </c>
       <c r="Y2" s="1">
-        <v>11.19</v>
+        <v>0.2238</v>
       </c>
       <c r="Z2" s="1">
-        <v>11.39</v>
+        <v>0.2278</v>
       </c>
       <c r="AA2" s="1">
-        <v>11.54</v>
+        <v>0.23079999999999998</v>
       </c>
       <c r="AB2" s="1">
-        <v>11.42</v>
+        <v>0.22839999999999999</v>
       </c>
       <c r="AC2" s="1">
-        <v>11.23</v>
+        <v>0.22460000000000002</v>
       </c>
     </row>
     <row r="3" spans="2:29" x14ac:dyDescent="0.3">
@@ -831,79 +831,79 @@
         <v>53</v>
       </c>
       <c r="C3" s="1">
-        <v>132.23904999999999</v>
+        <v>1.3213999999999999</v>
       </c>
       <c r="D3" s="1">
-        <v>131.3015</v>
+        <v>1.6412687500000001</v>
       </c>
       <c r="E3" s="1">
-        <v>131.93055000000001</v>
+        <v>1.6491318750000001</v>
       </c>
       <c r="F3" s="1">
-        <v>129.74175</v>
+        <v>1.6217718749999999</v>
       </c>
       <c r="G3" s="1">
-        <v>127.55155000000001</v>
+        <v>1.594394375</v>
       </c>
       <c r="H3" s="1">
-        <v>126.65445</v>
+        <v>1.583180625</v>
       </c>
       <c r="I3" s="1">
-        <v>126.69204999999999</v>
+        <v>1.583650625</v>
       </c>
       <c r="J3" s="1">
-        <v>126.2968</v>
+        <v>1.5787100000000001</v>
       </c>
       <c r="K3" s="1">
-        <v>135.67179999999999</v>
+        <v>1.6958974999999998</v>
       </c>
       <c r="L3" s="1">
-        <v>135.8202</v>
+        <v>1.6977525</v>
       </c>
       <c r="M3" s="1">
-        <v>136.5044</v>
+        <v>1.706305</v>
       </c>
       <c r="N3" s="1">
-        <v>136.34155000000001</v>
+        <v>1.7042693750000002</v>
       </c>
       <c r="Q3" t="s">
         <v>74</v>
       </c>
       <c r="R3" s="1">
-        <v>27.08</v>
+        <v>0.54159999999999997</v>
       </c>
       <c r="S3" s="1">
-        <v>26.59</v>
+        <v>0.53180000000000005</v>
       </c>
       <c r="T3" s="1">
-        <v>26.56</v>
+        <v>0.53120000000000001</v>
       </c>
       <c r="U3" s="1">
-        <v>26.43</v>
+        <v>0.52859999999999996</v>
       </c>
       <c r="V3" s="1">
-        <v>26.53</v>
+        <v>0.53060000000000007</v>
       </c>
       <c r="W3" s="1">
-        <v>26.62</v>
+        <v>0.53239999999999998</v>
       </c>
       <c r="X3" s="1">
-        <v>28.64</v>
+        <v>0.57279999999999998</v>
       </c>
       <c r="Y3" s="1">
-        <v>28.48</v>
+        <v>0.5696</v>
       </c>
       <c r="Z3" s="1">
-        <v>28.49</v>
+        <v>0.56979999999999997</v>
       </c>
       <c r="AA3" s="1">
-        <v>28.36</v>
+        <v>0.56720000000000004</v>
       </c>
       <c r="AB3" s="1">
-        <v>28.33</v>
+        <v>0.56659999999999999</v>
       </c>
       <c r="AC3" s="1">
-        <v>28.33</v>
+        <v>0.56659999999999999</v>
       </c>
     </row>
     <row r="4" spans="2:29" x14ac:dyDescent="0.3">
@@ -911,79 +911,79 @@
         <v>54</v>
       </c>
       <c r="C4" s="1">
-        <v>98.697000000000003</v>
+        <v>1.2337125</v>
       </c>
       <c r="D4" s="1">
-        <v>98.123900000000006</v>
+        <v>1.2265487500000001</v>
       </c>
       <c r="E4" s="1">
-        <v>98.475999999999999</v>
+        <v>1.23095</v>
       </c>
       <c r="F4" s="1">
-        <v>96.935450000000003</v>
+        <v>1.211693125</v>
       </c>
       <c r="G4" s="1">
-        <v>95.306049999999999</v>
+        <v>0.87346000000000001</v>
       </c>
       <c r="H4" s="1">
-        <v>94.453550000000007</v>
+        <v>1.1806693750000001</v>
       </c>
       <c r="I4" s="1">
-        <v>94.437550000000002</v>
+        <v>1.1804693749999999</v>
       </c>
       <c r="J4" s="1">
-        <v>94.905299999999997</v>
+        <v>1.18631625</v>
       </c>
       <c r="K4" s="1">
-        <v>99.905299999999997</v>
+        <v>1.24881625</v>
       </c>
       <c r="L4" s="1">
-        <v>100.9494</v>
+        <v>1.2618674999999999</v>
       </c>
       <c r="M4" s="1">
-        <v>101.38195</v>
+        <v>1.267274375</v>
       </c>
       <c r="N4" s="1">
-        <v>101.29595</v>
+        <v>1.266199375</v>
       </c>
       <c r="Q4" t="s">
         <v>75</v>
       </c>
       <c r="R4" s="1">
-        <v>22.56</v>
+        <v>0.45119999999999999</v>
       </c>
       <c r="S4" s="1">
-        <v>21.81</v>
+        <v>0.43619999999999998</v>
       </c>
       <c r="T4" s="1">
-        <v>21.04</v>
+        <v>0.42080000000000001</v>
       </c>
       <c r="U4" s="1">
-        <v>22.67</v>
+        <v>0.45340000000000003</v>
       </c>
       <c r="V4" s="1">
-        <v>22.79</v>
+        <v>0.45579999999999998</v>
       </c>
       <c r="W4" s="1">
-        <v>22.03</v>
+        <v>0.44060000000000005</v>
       </c>
       <c r="X4" s="1">
-        <v>23.94</v>
+        <v>0.4788</v>
       </c>
       <c r="Y4" s="1">
-        <v>23.36</v>
+        <v>0.4672</v>
       </c>
       <c r="Z4" s="1">
-        <v>24.09</v>
+        <v>0.48180000000000001</v>
       </c>
       <c r="AA4" s="1">
-        <v>23.67</v>
+        <v>0.47340000000000004</v>
       </c>
       <c r="AB4" s="1">
-        <v>23.7</v>
+        <v>0.47399999999999998</v>
       </c>
       <c r="AC4" s="1">
-        <v>23.38</v>
+        <v>0.46759999999999996</v>
       </c>
     </row>
     <row r="5" spans="2:29" x14ac:dyDescent="0.3">
@@ -991,79 +991,79 @@
         <v>55</v>
       </c>
       <c r="C5" s="1">
-        <v>14.815</v>
+        <v>0.1851875</v>
       </c>
       <c r="D5" s="1">
-        <v>14.79</v>
+        <v>1.18438</v>
       </c>
       <c r="E5" s="1">
-        <v>14.81</v>
+        <v>0.18512500000000001</v>
       </c>
       <c r="F5" s="1">
-        <v>14.605</v>
+        <v>0.18256250000000002</v>
       </c>
       <c r="G5" s="1">
-        <v>14.425000000000001</v>
+        <v>0.18031250000000001</v>
       </c>
       <c r="H5" s="1">
-        <v>14.555</v>
+        <v>0.1819375</v>
       </c>
       <c r="I5" s="1">
-        <v>14.25</v>
+        <v>0.17812500000000001</v>
       </c>
       <c r="J5" s="1">
-        <v>13.73</v>
+        <v>0.171625</v>
       </c>
       <c r="K5" s="1">
-        <v>12.595000000000001</v>
+        <v>0.15743750000000001</v>
       </c>
       <c r="L5" s="1">
-        <v>11.5</v>
+        <v>0.14374999999999999</v>
       </c>
       <c r="M5" s="1">
-        <v>11.875</v>
+        <v>0.1484375</v>
       </c>
       <c r="N5" s="1">
-        <v>11.7</v>
+        <v>0.14624999999999999</v>
       </c>
       <c r="Q5" t="s">
         <v>76</v>
       </c>
       <c r="R5" s="1">
-        <v>25.43</v>
+        <v>0.50859999999999994</v>
       </c>
       <c r="S5" s="1">
-        <v>25.34</v>
+        <v>0.50680000000000003</v>
       </c>
       <c r="T5" s="1">
-        <v>25</v>
+        <v>0.5</v>
       </c>
       <c r="U5" s="1">
-        <v>25.27</v>
+        <v>0.50539999999999996</v>
       </c>
       <c r="V5" s="1">
-        <v>25.52</v>
+        <v>0.51039999999999996</v>
       </c>
       <c r="W5" s="1">
-        <v>26.29</v>
+        <v>0.52579999999999993</v>
       </c>
       <c r="X5" s="1">
-        <v>28.1</v>
+        <v>0.56200000000000006</v>
       </c>
       <c r="Y5" s="1">
-        <v>29.57</v>
+        <v>0.59140000000000004</v>
       </c>
       <c r="Z5" s="1">
-        <v>30.99</v>
+        <v>0.61980000000000002</v>
       </c>
       <c r="AA5" s="1">
-        <v>30.54</v>
+        <v>0.61080000000000001</v>
       </c>
       <c r="AB5" s="1">
-        <v>30.57</v>
+        <v>0.61140000000000005</v>
       </c>
       <c r="AC5" s="1">
-        <v>30.22</v>
+        <v>0.60439999999999994</v>
       </c>
     </row>
     <row r="6" spans="2:29" x14ac:dyDescent="0.3">
@@ -1071,79 +1071,79 @@
         <v>56</v>
       </c>
       <c r="C6" s="1">
-        <v>22.08</v>
+        <v>0.27599999999999997</v>
       </c>
       <c r="D6" s="1">
-        <v>21.85</v>
+        <v>0.27312500000000001</v>
       </c>
       <c r="E6" s="1">
-        <v>21.975000000000001</v>
+        <v>0.27468750000000003</v>
       </c>
       <c r="F6" s="1">
-        <v>20.114999999999998</v>
+        <v>0.25143749999999998</v>
       </c>
       <c r="G6" s="1">
-        <v>23.66</v>
+        <v>1.09345</v>
       </c>
       <c r="H6" s="1">
-        <v>19.52</v>
+        <v>0.24399999999999999</v>
       </c>
       <c r="I6" s="1">
-        <v>17.41</v>
+        <v>0.21762500000000001</v>
       </c>
       <c r="J6" s="1">
-        <v>12.63</v>
+        <v>0.15787500000000002</v>
       </c>
       <c r="K6" s="1">
-        <v>12.775</v>
+        <v>0.15968750000000001</v>
       </c>
       <c r="L6" s="1">
-        <v>13.59</v>
+        <v>0.169875</v>
       </c>
       <c r="M6" s="1">
-        <v>11.734999999999999</v>
+        <v>0.1466875</v>
       </c>
       <c r="N6" s="1">
-        <v>14.994999999999999</v>
+        <v>0.18743749999999998</v>
       </c>
       <c r="Q6" t="s">
         <v>77</v>
       </c>
       <c r="R6" s="1">
-        <v>26.89</v>
+        <v>0.53780000000000006</v>
       </c>
       <c r="S6" s="1">
-        <v>27.2</v>
+        <v>0.78949999999999998</v>
       </c>
       <c r="T6" s="1">
-        <v>27.49</v>
+        <v>0.54979999999999996</v>
       </c>
       <c r="U6" s="1">
-        <v>29.53</v>
+        <v>0.59060000000000001</v>
       </c>
       <c r="V6" s="1">
-        <v>29.68</v>
+        <v>0.59360000000000002</v>
       </c>
       <c r="W6" s="1">
-        <v>31.23</v>
+        <v>0.62460000000000004</v>
       </c>
       <c r="X6" s="1">
-        <v>32.369999999999997</v>
+        <v>0.64739999999999998</v>
       </c>
       <c r="Y6" s="1">
-        <v>32.9</v>
+        <v>0.65799999999999992</v>
       </c>
       <c r="Z6" s="1">
-        <v>33.81</v>
+        <v>0.67620000000000002</v>
       </c>
       <c r="AA6" s="1">
-        <v>33.28</v>
+        <v>0.66559999999999997</v>
       </c>
       <c r="AB6" s="1">
-        <v>33.32</v>
+        <v>0.66639999999999999</v>
       </c>
       <c r="AC6" s="1">
-        <v>32.92</v>
+        <v>0.65839999999999999</v>
       </c>
     </row>
     <row r="7" spans="2:29" x14ac:dyDescent="0.3">
@@ -1151,79 +1151,79 @@
         <v>57</v>
       </c>
       <c r="C7" s="1">
-        <v>21.9</v>
+        <v>0.27374999999999999</v>
       </c>
       <c r="D7" s="1">
-        <v>21.105</v>
+        <v>1.2634000000000001</v>
       </c>
       <c r="E7" s="1">
-        <v>21.164999999999999</v>
+        <v>0.26456249999999998</v>
       </c>
       <c r="F7" s="1">
-        <v>23.925000000000001</v>
+        <v>0.29906250000000001</v>
       </c>
       <c r="G7" s="1">
-        <v>24.86</v>
+        <v>0.31074999999999997</v>
       </c>
       <c r="H7" s="1">
-        <v>25.03</v>
+        <v>1.3472900000000001</v>
       </c>
       <c r="I7" s="1">
-        <v>24.89</v>
+        <v>0.31112499999999998</v>
       </c>
       <c r="J7" s="1">
-        <v>24.09</v>
+        <v>0.30112499999999998</v>
       </c>
       <c r="K7" s="1">
-        <v>23.69</v>
+        <v>0.29612500000000003</v>
       </c>
       <c r="L7" s="1">
-        <v>22.925000000000001</v>
+        <v>1.1234329999999999</v>
       </c>
       <c r="M7" s="1">
-        <v>23.504999999999999</v>
+        <v>0.29381249999999998</v>
       </c>
       <c r="N7" s="1">
-        <v>23.23</v>
+        <v>0.29037499999999999</v>
       </c>
       <c r="Q7" t="s">
         <v>78</v>
       </c>
       <c r="R7" s="1">
-        <v>31.49</v>
+        <v>0.62979999999999992</v>
       </c>
       <c r="S7" s="1">
-        <v>31.74</v>
+        <v>0.63479999999999992</v>
       </c>
       <c r="T7" s="1">
-        <v>31.97</v>
+        <v>0.63939999999999997</v>
       </c>
       <c r="U7" s="1">
-        <v>32.61</v>
+        <v>0.6522</v>
       </c>
       <c r="V7" s="1">
-        <v>33.72</v>
+        <v>0.6744</v>
       </c>
       <c r="W7" s="1">
-        <v>34.97</v>
+        <v>0.69940000000000002</v>
       </c>
       <c r="X7" s="1">
-        <v>35.880000000000003</v>
+        <v>0.71760000000000002</v>
       </c>
       <c r="Y7" s="1">
-        <v>35.299999999999997</v>
+        <v>0.70599999999999996</v>
       </c>
       <c r="Z7" s="1">
-        <v>36.020000000000003</v>
+        <v>0.72040000000000004</v>
       </c>
       <c r="AA7" s="1">
-        <v>36.61</v>
+        <v>0.73219999999999996</v>
       </c>
       <c r="AB7" s="1">
-        <v>36.64</v>
+        <v>0.73280000000000001</v>
       </c>
       <c r="AC7" s="1">
-        <v>36.31</v>
+        <v>0.72620000000000007</v>
       </c>
     </row>
     <row r="8" spans="2:29" x14ac:dyDescent="0.3">
@@ -1231,79 +1231,79 @@
         <v>58</v>
       </c>
       <c r="C8" s="1">
-        <v>16.899999999999999</v>
+        <v>0.21124999999999999</v>
       </c>
       <c r="D8" s="1">
-        <v>16.105</v>
+        <v>0.20131250000000001</v>
       </c>
       <c r="E8" s="1">
-        <v>16.164999999999999</v>
+        <v>0.20206249999999998</v>
       </c>
       <c r="F8" s="1">
-        <v>18.925000000000001</v>
+        <v>0.23656250000000001</v>
       </c>
       <c r="G8" s="1">
-        <v>19.86</v>
+        <v>0.24825</v>
       </c>
       <c r="H8" s="1">
-        <v>20.03</v>
+        <v>0.48324</v>
       </c>
       <c r="I8" s="1">
-        <v>19.89</v>
+        <v>1.2387600000000001</v>
       </c>
       <c r="J8" s="1">
-        <v>19.09</v>
+        <v>0.238625</v>
       </c>
       <c r="K8" s="1">
-        <v>18.690000000000001</v>
+        <v>0.98763000000000001</v>
       </c>
       <c r="L8" s="1">
-        <v>17.925000000000001</v>
+        <v>0.2240625</v>
       </c>
       <c r="M8" s="1">
-        <v>18.504999999999999</v>
+        <v>0.23131249999999998</v>
       </c>
       <c r="N8" s="1">
-        <v>18.23</v>
+        <v>0.98363</v>
       </c>
       <c r="Q8" t="s">
         <v>79</v>
       </c>
       <c r="R8" s="1">
-        <v>35.18</v>
+        <v>0.7036</v>
       </c>
       <c r="S8" s="1">
-        <v>33.72</v>
+        <v>0.6744</v>
       </c>
       <c r="T8" s="1">
-        <v>33.08</v>
+        <v>0.66159999999999997</v>
       </c>
       <c r="U8" s="1">
-        <v>33.4</v>
+        <v>0.66799999999999993</v>
       </c>
       <c r="V8" s="1">
-        <v>33.72</v>
+        <v>0.6744</v>
       </c>
       <c r="W8" s="1">
-        <v>35.880000000000003</v>
+        <v>0.71760000000000002</v>
       </c>
       <c r="X8" s="1">
-        <v>34.630000000000003</v>
+        <v>0.6926000000000001</v>
       </c>
       <c r="Y8" s="1">
-        <v>35.93</v>
+        <v>0.71860000000000002</v>
       </c>
       <c r="Z8" s="1">
-        <v>36.56</v>
+        <v>0.73120000000000007</v>
       </c>
       <c r="AA8" s="1">
-        <v>37.97</v>
+        <v>0.75939999999999996</v>
       </c>
       <c r="AB8" s="1">
-        <v>36.01</v>
+        <v>0.72019999999999995</v>
       </c>
       <c r="AC8" s="1">
-        <v>36.549999999999997</v>
+        <v>0.73099999999999998</v>
       </c>
     </row>
     <row r="9" spans="2:29" x14ac:dyDescent="0.3">
@@ -1311,79 +1311,79 @@
         <v>59</v>
       </c>
       <c r="C9" s="1">
-        <v>40.064999999999998</v>
+        <v>0.50081249999999999</v>
       </c>
       <c r="D9" s="1">
-        <v>40.79</v>
+        <v>0.50987499999999997</v>
       </c>
       <c r="E9" s="1">
-        <v>40.26</v>
+        <v>0.94723999999999997</v>
       </c>
       <c r="F9" s="1">
-        <v>40.805</v>
+        <v>0.51006249999999997</v>
       </c>
       <c r="G9" s="1">
-        <v>42.274999999999999</v>
+        <v>0.5284375</v>
       </c>
       <c r="H9" s="1">
-        <v>39.655000000000001</v>
+        <v>0.4956875</v>
       </c>
       <c r="I9" s="1">
-        <v>39.75</v>
+        <v>0.49687500000000001</v>
       </c>
       <c r="J9" s="1">
-        <v>39.229999999999997</v>
+        <v>0.49037499999999995</v>
       </c>
       <c r="K9" s="1">
-        <v>38.094999999999999</v>
+        <v>0.98364300000000005</v>
       </c>
       <c r="L9" s="1">
-        <v>37.049999999999997</v>
+        <v>1.7632300000000001</v>
       </c>
       <c r="M9" s="1">
-        <v>37.024999999999999</v>
+        <v>1.46322</v>
       </c>
       <c r="N9" s="1">
-        <v>37.299999999999997</v>
+        <v>0.46624999999999994</v>
       </c>
       <c r="Q9" t="s">
         <v>80</v>
       </c>
       <c r="R9" s="1">
-        <v>84.47</v>
+        <v>1.6894</v>
       </c>
       <c r="S9" s="1">
-        <v>84.72</v>
+        <v>1.6943999999999999</v>
       </c>
       <c r="T9" s="1">
-        <v>84.95</v>
+        <v>1.6990000000000001</v>
       </c>
       <c r="U9" s="1">
-        <v>86.59</v>
+        <v>1.7318</v>
       </c>
       <c r="V9" s="1">
-        <v>86.7</v>
+        <v>1.734</v>
       </c>
       <c r="W9" s="1">
-        <v>87.94</v>
+        <v>1.7587999999999999</v>
       </c>
       <c r="X9" s="1">
-        <v>88</v>
+        <v>1.76</v>
       </c>
       <c r="Y9" s="1">
-        <v>89.58</v>
+        <v>1.7915999999999999</v>
       </c>
       <c r="Z9" s="1">
-        <v>88.62</v>
+        <v>1.7724000000000002</v>
       </c>
       <c r="AA9" s="1">
-        <v>89.29</v>
+        <v>1.2464999999999999</v>
       </c>
       <c r="AB9" s="1">
-        <v>88.71</v>
+        <v>1.7741999999999998</v>
       </c>
       <c r="AC9" s="1">
-        <v>89.23</v>
+        <v>1.7846000000000002</v>
       </c>
     </row>
     <row r="10" spans="2:29" x14ac:dyDescent="0.3">
@@ -1391,79 +1391,79 @@
         <v>60</v>
       </c>
       <c r="C10" s="1">
-        <v>2.9</v>
+        <v>3.6249999999999998E-2</v>
       </c>
       <c r="D10" s="1">
-        <v>2.605</v>
+        <v>3.2562500000000001E-2</v>
       </c>
       <c r="E10" s="1">
-        <v>2.665</v>
+        <v>3.3312500000000002E-2</v>
       </c>
       <c r="F10" s="1">
-        <v>2.9249999999999998</v>
+        <v>3.6562499999999998E-2</v>
       </c>
       <c r="G10" s="1">
-        <v>2.86</v>
+        <v>3.5749999999999997E-2</v>
       </c>
       <c r="H10" s="1">
-        <v>2.5299999999999998</v>
+        <v>3.1625E-2</v>
       </c>
       <c r="I10" s="1">
-        <v>2.89</v>
+        <v>1.1984300000000001</v>
       </c>
       <c r="J10" s="1">
-        <v>2.59</v>
+        <v>3.2375000000000001E-2</v>
       </c>
       <c r="K10" s="1">
-        <v>2.69</v>
+        <v>3.3625000000000002E-2</v>
       </c>
       <c r="L10" s="1">
-        <v>2.9249999999999998</v>
+        <v>3.6562499999999998E-2</v>
       </c>
       <c r="M10" s="1">
-        <v>2.5049999999999999</v>
+        <v>3.13125E-2</v>
       </c>
       <c r="N10" s="1">
-        <v>2.73</v>
+        <v>3.4125000000000003E-2</v>
       </c>
       <c r="Q10" t="s">
         <v>81</v>
       </c>
       <c r="R10" s="1">
-        <v>13.54</v>
+        <v>0.27079999999999999</v>
       </c>
       <c r="S10" s="1">
-        <v>13.63</v>
+        <v>0.27260000000000001</v>
       </c>
       <c r="T10" s="1">
-        <v>13.71</v>
+        <v>0.2742</v>
       </c>
       <c r="U10" s="1">
-        <v>14.27</v>
+        <v>0.28539999999999999</v>
       </c>
       <c r="V10" s="1">
-        <v>14.31</v>
+        <v>0.28620000000000001</v>
       </c>
       <c r="W10" s="1">
-        <v>14.74</v>
+        <v>0.29480000000000001</v>
       </c>
       <c r="X10" s="1">
-        <v>15.45</v>
+        <v>0.309</v>
       </c>
       <c r="Y10" s="1">
-        <v>15.3</v>
+        <v>0.30599999999999999</v>
       </c>
       <c r="Z10" s="1">
-        <v>15.31</v>
+        <v>0.30620000000000003</v>
       </c>
       <c r="AA10" s="1">
-        <v>15.2</v>
+        <v>0.30399999999999999</v>
       </c>
       <c r="AB10" s="1">
-        <v>15.17</v>
+        <v>0.3034</v>
       </c>
       <c r="AC10" s="1">
-        <v>15.18</v>
+        <v>0.30359999999999998</v>
       </c>
     </row>
     <row r="11" spans="2:29" x14ac:dyDescent="0.3">
@@ -1471,79 +1471,79 @@
         <v>61</v>
       </c>
       <c r="C11" s="1">
-        <v>2.9</v>
+        <v>3.6249999999999998E-2</v>
       </c>
       <c r="D11" s="1">
-        <v>2.605</v>
+        <v>3.2562500000000001E-2</v>
       </c>
       <c r="E11" s="1">
-        <v>2.665</v>
+        <v>3.3312500000000002E-2</v>
       </c>
       <c r="F11" s="1">
-        <v>2.9249999999999998</v>
+        <v>3.6562499999999998E-2</v>
       </c>
       <c r="G11" s="1">
-        <v>2.86</v>
+        <v>3.5749999999999997E-2</v>
       </c>
       <c r="H11" s="1">
-        <v>2.5299999999999998</v>
+        <v>3.1625E-2</v>
       </c>
       <c r="I11" s="1">
-        <v>2.89</v>
+        <v>3.6125000000000004E-2</v>
       </c>
       <c r="J11" s="1">
-        <v>2.59</v>
+        <v>3.2375000000000001E-2</v>
       </c>
       <c r="K11" s="1">
-        <v>2.69</v>
+        <v>3.3625000000000002E-2</v>
       </c>
       <c r="L11" s="1">
-        <v>2.9249999999999998</v>
+        <v>3.6562499999999998E-2</v>
       </c>
       <c r="M11" s="1">
-        <v>2.5049999999999999</v>
+        <v>3.13125E-2</v>
       </c>
       <c r="N11" s="1">
-        <v>2.73</v>
+        <v>1.3948472999999999</v>
       </c>
       <c r="Q11" t="s">
         <v>82</v>
       </c>
       <c r="R11" s="1">
-        <v>26.89</v>
+        <v>0.53780000000000006</v>
       </c>
       <c r="S11" s="1">
-        <v>27.2</v>
+        <v>0.54400000000000004</v>
       </c>
       <c r="T11" s="1">
-        <v>27.49</v>
+        <v>0.54979999999999996</v>
       </c>
       <c r="U11" s="1">
-        <v>29.53</v>
+        <v>0.59060000000000001</v>
       </c>
       <c r="V11" s="1">
-        <v>29.68</v>
+        <v>0.59360000000000002</v>
       </c>
       <c r="W11" s="1">
-        <v>31.23</v>
+        <v>0.62460000000000004</v>
       </c>
       <c r="X11" s="1">
-        <v>32.369999999999997</v>
+        <v>0.64739999999999998</v>
       </c>
       <c r="Y11" s="1">
-        <v>32.9</v>
+        <v>0.65799999999999992</v>
       </c>
       <c r="Z11" s="1">
-        <v>33.81</v>
+        <v>0.67620000000000002</v>
       </c>
       <c r="AA11" s="1">
-        <v>33.28</v>
+        <v>0.66559999999999997</v>
       </c>
       <c r="AB11" s="1">
-        <v>33.32</v>
+        <v>0.66639999999999999</v>
       </c>
       <c r="AC11" s="1">
-        <v>32.92</v>
+        <v>0.65839999999999999</v>
       </c>
     </row>
     <row r="12" spans="2:29" x14ac:dyDescent="0.3">
@@ -1551,79 +1551,79 @@
         <v>62</v>
       </c>
       <c r="C12" s="1">
-        <v>40.064999999999998</v>
+        <v>0.50081249999999999</v>
       </c>
       <c r="D12" s="1">
-        <v>40.79</v>
+        <v>0.50987499999999997</v>
       </c>
       <c r="E12" s="1">
-        <v>40.26</v>
+        <v>0.50324999999999998</v>
       </c>
       <c r="F12" s="1">
-        <v>40.805</v>
+        <v>0.51006249999999997</v>
       </c>
       <c r="G12" s="1">
-        <v>42.274999999999999</v>
+        <v>0.5284375</v>
       </c>
       <c r="H12" s="1">
-        <v>39.655000000000001</v>
+        <v>0.4956875</v>
       </c>
       <c r="I12" s="1">
-        <v>39.75</v>
+        <v>0.49687500000000001</v>
       </c>
       <c r="J12" s="1">
-        <v>39.229999999999997</v>
+        <v>1.4928269999999999</v>
       </c>
       <c r="K12" s="1">
-        <v>38.094999999999999</v>
+        <v>0.98476432999999997</v>
       </c>
       <c r="L12" s="1">
-        <v>37.049999999999997</v>
+        <v>0.46312499999999995</v>
       </c>
       <c r="M12" s="1">
-        <v>37.024999999999999</v>
+        <v>0.46281249999999996</v>
       </c>
       <c r="N12" s="1">
-        <v>37.299999999999997</v>
+        <v>0.46624999999999994</v>
       </c>
       <c r="Q12" t="s">
         <v>83</v>
       </c>
       <c r="R12" s="1">
-        <v>31.49</v>
+        <v>0.62979999999999992</v>
       </c>
       <c r="S12" s="1">
-        <v>31.74</v>
+        <v>0.63479999999999992</v>
       </c>
       <c r="T12" s="1">
-        <v>31.97</v>
+        <v>0.63939999999999997</v>
       </c>
       <c r="U12" s="1">
-        <v>32.61</v>
+        <v>0.6522</v>
       </c>
       <c r="V12" s="1">
-        <v>33.72</v>
+        <v>0.6744</v>
       </c>
       <c r="W12" s="1">
-        <v>34.97</v>
+        <v>0.69940000000000002</v>
       </c>
       <c r="X12" s="1">
-        <v>35.880000000000003</v>
+        <v>0.71760000000000002</v>
       </c>
       <c r="Y12" s="1">
-        <v>35.299999999999997</v>
+        <v>0.70599999999999996</v>
       </c>
       <c r="Z12" s="1">
-        <v>36.020000000000003</v>
+        <v>0.72040000000000004</v>
       </c>
       <c r="AA12" s="1">
-        <v>36.61</v>
+        <v>0.73219999999999996</v>
       </c>
       <c r="AB12" s="1">
-        <v>36.64</v>
+        <v>0.73280000000000001</v>
       </c>
       <c r="AC12" s="1">
-        <v>36.31</v>
+        <v>0.72620000000000007</v>
       </c>
     </row>
     <row r="13" spans="2:29" x14ac:dyDescent="0.3">
@@ -1631,79 +1631,79 @@
         <v>63</v>
       </c>
       <c r="C13" s="1">
-        <v>16.899999999999999</v>
+        <v>0.21124999999999999</v>
       </c>
       <c r="D13" s="1">
-        <v>16.105</v>
+        <v>0.20131250000000001</v>
       </c>
       <c r="E13" s="1">
-        <v>16.164999999999999</v>
+        <v>0.20206249999999998</v>
       </c>
       <c r="F13" s="1">
-        <v>18.925000000000001</v>
+        <v>0.23656250000000001</v>
       </c>
       <c r="G13" s="1">
-        <v>19.86</v>
+        <v>0.24825</v>
       </c>
       <c r="H13" s="1">
-        <v>20.03</v>
+        <v>0.25037500000000001</v>
       </c>
       <c r="I13" s="1">
-        <v>19.89</v>
+        <v>0.24862500000000001</v>
       </c>
       <c r="J13" s="1">
-        <v>19.09</v>
+        <v>0.238625</v>
       </c>
       <c r="K13" s="1">
-        <v>18.690000000000001</v>
+        <v>0.23362500000000003</v>
       </c>
       <c r="L13" s="1">
-        <v>17.925000000000001</v>
+        <v>0.2240625</v>
       </c>
       <c r="M13" s="1">
-        <v>18.504999999999999</v>
+        <v>1.3434984999999999</v>
       </c>
       <c r="N13" s="1">
-        <v>18.23</v>
+        <v>0.22787499999999999</v>
       </c>
       <c r="Q13" t="s">
         <v>84</v>
       </c>
       <c r="R13" s="1">
-        <v>35.18</v>
+        <v>0.7036</v>
       </c>
       <c r="S13" s="1">
-        <v>33.72</v>
+        <v>0.6744</v>
       </c>
       <c r="T13" s="1">
-        <v>33.08</v>
+        <v>0.66159999999999997</v>
       </c>
       <c r="U13" s="1">
-        <v>33.4</v>
+        <v>0.66799999999999993</v>
       </c>
       <c r="V13" s="1">
-        <v>33.72</v>
+        <v>0.6744</v>
       </c>
       <c r="W13" s="1">
-        <v>35.880000000000003</v>
+        <v>0.71760000000000002</v>
       </c>
       <c r="X13" s="1">
-        <v>34.630000000000003</v>
+        <v>0.6926000000000001</v>
       </c>
       <c r="Y13" s="1">
-        <v>35.93</v>
+        <v>0.71860000000000002</v>
       </c>
       <c r="Z13" s="1">
-        <v>36.56</v>
+        <v>0.73120000000000007</v>
       </c>
       <c r="AA13" s="1">
-        <v>37.97</v>
+        <v>0.75939999999999996</v>
       </c>
       <c r="AB13" s="1">
-        <v>36.01</v>
+        <v>0.72019999999999995</v>
       </c>
       <c r="AC13" s="1">
-        <v>36.549999999999997</v>
+        <v>0.73099999999999998</v>
       </c>
     </row>
     <row r="14" spans="2:29" x14ac:dyDescent="0.3">
@@ -1711,79 +1711,79 @@
         <v>64</v>
       </c>
       <c r="C14" s="1">
-        <v>21.9</v>
+        <v>0.27374999999999999</v>
       </c>
       <c r="D14" s="1">
-        <v>21.105</v>
+        <v>0.26381250000000001</v>
       </c>
       <c r="E14" s="1">
-        <v>21.164999999999999</v>
+        <v>0.26456249999999998</v>
       </c>
       <c r="F14" s="1">
-        <v>23.925000000000001</v>
+        <v>0.29906250000000001</v>
       </c>
       <c r="G14" s="1">
-        <v>24.86</v>
+        <v>0.31074999999999997</v>
       </c>
       <c r="H14" s="1">
-        <v>25.03</v>
+        <v>0.31287500000000001</v>
       </c>
       <c r="I14" s="1">
-        <v>24.89</v>
+        <v>0.31112499999999998</v>
       </c>
       <c r="J14" s="1">
-        <v>24.09</v>
+        <v>0.30112499999999998</v>
       </c>
       <c r="K14" s="1">
-        <v>23.69</v>
+        <v>0.29612500000000003</v>
       </c>
       <c r="L14" s="1">
-        <v>22.925000000000001</v>
+        <v>0.2865625</v>
       </c>
       <c r="M14" s="1">
-        <v>23.504999999999999</v>
+        <v>0.29381249999999998</v>
       </c>
       <c r="N14" s="1">
-        <v>23.23</v>
+        <v>0.29037499999999999</v>
       </c>
       <c r="Q14" t="s">
         <v>85</v>
       </c>
       <c r="R14" s="1">
-        <v>84.47</v>
+        <v>1.6894</v>
       </c>
       <c r="S14" s="1">
-        <v>84.72</v>
+        <v>1.6943999999999999</v>
       </c>
       <c r="T14" s="1">
-        <v>84.95</v>
+        <v>1.6990000000000001</v>
       </c>
       <c r="U14" s="1">
-        <v>86.59</v>
+        <v>1.7318</v>
       </c>
       <c r="V14" s="1">
-        <v>86.7</v>
+        <v>1.734</v>
       </c>
       <c r="W14" s="1">
-        <v>87.94</v>
+        <v>1.7587999999999999</v>
       </c>
       <c r="X14" s="1">
-        <v>88</v>
+        <v>1.76</v>
       </c>
       <c r="Y14" s="1">
-        <v>89.58</v>
+        <v>1.7915999999999999</v>
       </c>
       <c r="Z14" s="1">
-        <v>88.62</v>
+        <v>1.7724000000000002</v>
       </c>
       <c r="AA14" s="1">
-        <v>89.29</v>
+        <v>1.7858000000000001</v>
       </c>
       <c r="AB14" s="1">
-        <v>88.71</v>
+        <v>1.7741999999999998</v>
       </c>
       <c r="AC14" s="1">
-        <v>89.23</v>
+        <v>1.7846000000000002</v>
       </c>
     </row>
     <row r="15" spans="2:29" x14ac:dyDescent="0.3">
@@ -1791,79 +1791,79 @@
         <v>65</v>
       </c>
       <c r="C15" s="1">
-        <v>22.08</v>
+        <v>0.27599999999999997</v>
       </c>
       <c r="D15" s="1">
-        <v>21.85</v>
+        <v>0.27312500000000001</v>
       </c>
       <c r="E15" s="1">
-        <v>21.975000000000001</v>
+        <v>0.27468750000000003</v>
       </c>
       <c r="F15" s="1">
-        <v>20.114999999999998</v>
+        <v>0.25143749999999998</v>
       </c>
       <c r="G15" s="1">
-        <v>23.66</v>
+        <v>0.29575000000000001</v>
       </c>
       <c r="H15" s="1">
-        <v>19.52</v>
+        <v>0.24399999999999999</v>
       </c>
       <c r="I15" s="1">
-        <v>17.41</v>
+        <v>0.21762500000000001</v>
       </c>
       <c r="J15" s="1">
-        <v>12.63</v>
+        <v>0.15787500000000002</v>
       </c>
       <c r="K15" s="1">
-        <v>12.775</v>
+        <v>0.15968750000000001</v>
       </c>
       <c r="L15" s="1">
-        <v>13.59</v>
+        <v>0.169875</v>
       </c>
       <c r="M15" s="1">
-        <v>11.734999999999999</v>
+        <v>0.1466875</v>
       </c>
       <c r="N15" s="1">
-        <v>14.994999999999999</v>
+        <v>0.18743749999999998</v>
       </c>
       <c r="Q15" t="s">
         <v>86</v>
       </c>
       <c r="R15" s="1">
-        <v>13.54</v>
+        <v>0.27079999999999999</v>
       </c>
       <c r="S15" s="1">
-        <v>13.63</v>
+        <v>0.27260000000000001</v>
       </c>
       <c r="T15" s="1">
-        <v>13.71</v>
+        <v>0.2742</v>
       </c>
       <c r="U15" s="1">
-        <v>14.27</v>
+        <v>0.28539999999999999</v>
       </c>
       <c r="V15" s="1">
-        <v>14.31</v>
+        <v>0.28620000000000001</v>
       </c>
       <c r="W15" s="1">
-        <v>14.74</v>
+        <v>0.29480000000000001</v>
       </c>
       <c r="X15" s="1">
-        <v>15.45</v>
+        <v>0.309</v>
       </c>
       <c r="Y15" s="1">
-        <v>15.3</v>
+        <v>0.30599999999999999</v>
       </c>
       <c r="Z15" s="1">
-        <v>15.31</v>
+        <v>0.30620000000000003</v>
       </c>
       <c r="AA15" s="1">
-        <v>15.2</v>
+        <v>0.30399999999999999</v>
       </c>
       <c r="AB15" s="1">
-        <v>15.17</v>
+        <v>0.3034</v>
       </c>
       <c r="AC15" s="1">
-        <v>15.18</v>
+        <v>0.30359999999999998</v>
       </c>
     </row>
     <row r="16" spans="2:29" x14ac:dyDescent="0.3">
@@ -1871,40 +1871,40 @@
         <v>66</v>
       </c>
       <c r="C16" s="1">
-        <v>14.815</v>
+        <v>0.1851875</v>
       </c>
       <c r="D16" s="1">
-        <v>14.79</v>
+        <v>0.18487499999999998</v>
       </c>
       <c r="E16" s="1">
-        <v>14.81</v>
+        <v>0.18512500000000001</v>
       </c>
       <c r="F16" s="1">
-        <v>14.605</v>
+        <v>0.18256250000000002</v>
       </c>
       <c r="G16" s="1">
-        <v>14.425000000000001</v>
+        <v>0.18031250000000001</v>
       </c>
       <c r="H16" s="1">
-        <v>14.555</v>
+        <v>0.1819375</v>
       </c>
       <c r="I16" s="1">
-        <v>14.25</v>
+        <v>0.17812500000000001</v>
       </c>
       <c r="J16" s="1">
-        <v>13.73</v>
+        <v>0.171625</v>
       </c>
       <c r="K16" s="1">
-        <v>12.595000000000001</v>
+        <v>1.2334400000000001</v>
       </c>
       <c r="L16" s="1">
-        <v>11.5</v>
+        <v>0.14374999999999999</v>
       </c>
       <c r="M16" s="1">
-        <v>11.875</v>
+        <v>1.292734</v>
       </c>
       <c r="N16" s="1">
-        <v>11.7</v>
+        <v>0.14624999999999999</v>
       </c>
     </row>
     <row r="17" spans="2:28" x14ac:dyDescent="0.3">
@@ -1912,40 +1912,40 @@
         <v>67</v>
       </c>
       <c r="C17" s="1">
-        <v>22.08</v>
+        <v>0.27599999999999997</v>
       </c>
       <c r="D17" s="1">
-        <v>21.85</v>
+        <v>0.27312500000000001</v>
       </c>
       <c r="E17" s="1">
-        <v>21.975000000000001</v>
+        <v>0.27468750000000003</v>
       </c>
       <c r="F17" s="1">
-        <v>20.114999999999998</v>
+        <v>0.25143749999999998</v>
       </c>
       <c r="G17" s="1">
-        <v>23.66</v>
+        <v>0.29575000000000001</v>
       </c>
       <c r="H17" s="1">
-        <v>19.52</v>
+        <v>0.24399999999999999</v>
       </c>
       <c r="I17" s="1">
-        <v>17.41</v>
+        <v>0.21762500000000001</v>
       </c>
       <c r="J17" s="1">
-        <v>12.63</v>
+        <v>1.2364299999999999</v>
       </c>
       <c r="K17" s="1">
-        <v>12.775</v>
+        <v>0.15968750000000001</v>
       </c>
       <c r="L17" s="1">
-        <v>13.59</v>
+        <v>0.169875</v>
       </c>
       <c r="M17" s="1">
-        <v>11.734999999999999</v>
+        <v>0.1466875</v>
       </c>
       <c r="N17" s="1">
-        <v>14.994999999999999</v>
+        <v>1.2774939999999999</v>
       </c>
       <c r="X17" t="s">
         <v>87</v>
@@ -1956,40 +1956,40 @@
         <v>68</v>
       </c>
       <c r="C18" s="1">
-        <v>40.064999999999998</v>
+        <v>0.50081249999999999</v>
       </c>
       <c r="D18" s="1">
-        <v>40.79</v>
+        <v>0.50987499999999997</v>
       </c>
       <c r="E18" s="1">
-        <v>40.26</v>
+        <v>0.50324999999999998</v>
       </c>
       <c r="F18" s="1">
-        <v>40.805</v>
+        <v>0.51006249999999997</v>
       </c>
       <c r="G18" s="1">
-        <v>42.274999999999999</v>
+        <v>0.5284375</v>
       </c>
       <c r="H18" s="1">
-        <v>39.655000000000001</v>
+        <v>0.4956875</v>
       </c>
       <c r="I18" s="1">
-        <v>39.75</v>
+        <v>0.49687500000000001</v>
       </c>
       <c r="J18" s="1">
-        <v>39.229999999999997</v>
+        <v>0.49037499999999995</v>
       </c>
       <c r="K18" s="1">
-        <v>38.094999999999999</v>
+        <v>0.47618749999999999</v>
       </c>
       <c r="L18" s="1">
-        <v>37.049999999999997</v>
+        <v>0.46312499999999995</v>
       </c>
       <c r="M18" s="1">
-        <v>37.024999999999999</v>
+        <v>0.46281249999999996</v>
       </c>
       <c r="N18" s="1">
-        <v>37.299999999999997</v>
+        <v>0.46624999999999994</v>
       </c>
     </row>
     <row r="19" spans="2:28" x14ac:dyDescent="0.3">
@@ -1997,40 +1997,40 @@
         <v>69</v>
       </c>
       <c r="C19" s="1">
-        <v>16.899999999999999</v>
+        <v>0.21124999999999999</v>
       </c>
       <c r="D19" s="1">
-        <v>16.105</v>
+        <v>0.20131250000000001</v>
       </c>
       <c r="E19" s="1">
-        <v>16.164999999999999</v>
+        <v>0.20206249999999998</v>
       </c>
       <c r="F19" s="1">
-        <v>18.925000000000001</v>
+        <v>0.23656250000000001</v>
       </c>
       <c r="G19" s="1">
-        <v>19.86</v>
+        <v>0.24825</v>
       </c>
       <c r="H19" s="1">
-        <v>20.03</v>
+        <v>0.25037500000000001</v>
       </c>
       <c r="I19" s="1">
-        <v>19.89</v>
+        <v>0.24862500000000001</v>
       </c>
       <c r="J19" s="1">
-        <v>19.09</v>
+        <v>0.238625</v>
       </c>
       <c r="K19" s="1">
-        <v>18.690000000000001</v>
+        <v>1.2384299999999999</v>
       </c>
       <c r="L19" s="1">
-        <v>17.925000000000001</v>
+        <v>0.2240625</v>
       </c>
       <c r="M19" s="1">
-        <v>18.504999999999999</v>
+        <v>0.23131249999999998</v>
       </c>
       <c r="N19" s="1">
-        <v>18.23</v>
+        <v>0.22787499999999999</v>
       </c>
     </row>
     <row r="20" spans="2:28" x14ac:dyDescent="0.3">
@@ -2038,40 +2038,40 @@
         <v>70</v>
       </c>
       <c r="C20" s="1">
-        <v>21.9</v>
+        <v>0.27374999999999999</v>
       </c>
       <c r="D20" s="1">
-        <v>21.105</v>
+        <v>0.26381250000000001</v>
       </c>
       <c r="E20" s="1">
-        <v>21.164999999999999</v>
+        <v>0.26456249999999998</v>
       </c>
       <c r="F20" s="1">
-        <v>23.925000000000001</v>
+        <v>0.29906250000000001</v>
       </c>
       <c r="G20" s="1">
-        <v>24.86</v>
+        <v>0.31074999999999997</v>
       </c>
       <c r="H20" s="1">
-        <v>25.03</v>
+        <v>0.31287500000000001</v>
       </c>
       <c r="I20" s="1">
-        <v>24.89</v>
+        <v>0.31112499999999998</v>
       </c>
       <c r="J20" s="1">
-        <v>24.09</v>
+        <v>0.978634</v>
       </c>
       <c r="K20" s="1">
-        <v>23.69</v>
+        <v>0.29612500000000003</v>
       </c>
       <c r="L20" s="1">
-        <v>22.925000000000001</v>
+        <v>0.2865625</v>
       </c>
       <c r="M20" s="1">
-        <v>23.504999999999999</v>
+        <v>0.29381249999999998</v>
       </c>
       <c r="N20" s="1">
-        <v>23.23</v>
+        <v>0.29037499999999999</v>
       </c>
     </row>
     <row r="21" spans="2:28" x14ac:dyDescent="0.3">
@@ -2079,57 +2079,46 @@
         <v>71</v>
       </c>
       <c r="C21" s="1">
-        <v>2.9</v>
+        <v>3.6249999999999998E-2</v>
       </c>
       <c r="D21" s="1">
-        <v>2.605</v>
+        <v>3.2562500000000001E-2</v>
       </c>
       <c r="E21" s="1">
-        <v>2.665</v>
+        <v>3.3312500000000002E-2</v>
       </c>
       <c r="F21" s="1">
-        <v>2.9249999999999998</v>
+        <v>3.6562499999999998E-2</v>
       </c>
       <c r="G21" s="1">
-        <v>2.86</v>
+        <v>3.5749999999999997E-2</v>
       </c>
       <c r="H21" s="1">
-        <v>2.5299999999999998</v>
+        <v>3.1625E-2</v>
       </c>
       <c r="I21" s="1">
-        <v>2.89</v>
+        <v>3.6125000000000004E-2</v>
       </c>
       <c r="J21" s="1">
-        <v>2.59</v>
+        <v>3.2375000000000001E-2</v>
       </c>
       <c r="K21" s="1">
-        <v>2.69</v>
+        <v>3.3625000000000002E-2</v>
       </c>
       <c r="L21" s="1">
-        <v>2.9249999999999998</v>
+        <v>3.6562499999999998E-2</v>
       </c>
       <c r="M21" s="1">
-        <v>2.5049999999999999</v>
+        <v>1.2374430000000001</v>
       </c>
       <c r="N21" s="1">
-        <v>2.73</v>
-      </c>
-    </row>
-    <row r="22" spans="2:28" x14ac:dyDescent="0.3"/>
+        <v>1.2343500000000001</v>
+      </c>
+    </row>
     <row r="23" spans="2:28" x14ac:dyDescent="0.3">
       <c r="I23" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="24" spans="2:28" x14ac:dyDescent="0.3"/>
-    <row r="25" spans="2:28" x14ac:dyDescent="0.3"/>
-    <row r="26" spans="2:28" x14ac:dyDescent="0.3"/>
-    <row r="27" spans="2:28" x14ac:dyDescent="0.3"/>
-    <row r="28" spans="2:28" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="2:28" x14ac:dyDescent="0.3">
-      <c r="Z29" s="1"/>
-      <c r="AA29" s="1"/>
-      <c r="AB29" s="1"/>
     </row>
     <row r="30" spans="2:28" x14ac:dyDescent="0.3">
       <c r="Z30" s="1"/>
@@ -2145,76 +2134,6 @@
       <c r="Z32" s="1"/>
       <c r="AA32" s="1"/>
       <c r="AB32" s="1"/>
-    </row>
-    <row r="33" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z33" s="1"/>
-      <c r="AA33" s="1"/>
-      <c r="AB33" s="1"/>
-    </row>
-    <row r="34" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z34" s="1"/>
-      <c r="AA34" s="1"/>
-      <c r="AB34" s="1"/>
-    </row>
-    <row r="35" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z35" s="1"/>
-      <c r="AA35" s="1"/>
-      <c r="AB35" s="1"/>
-    </row>
-    <row r="36" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z36" s="1"/>
-      <c r="AA36" s="1"/>
-      <c r="AB36" s="1"/>
-    </row>
-    <row r="37" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z37" s="1"/>
-      <c r="AA37" s="1"/>
-      <c r="AB37" s="1"/>
-    </row>
-    <row r="38" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z38" s="1"/>
-      <c r="AA38" s="1"/>
-      <c r="AB38" s="1"/>
-    </row>
-    <row r="39" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z39" s="1"/>
-      <c r="AA39" s="1"/>
-      <c r="AB39" s="1"/>
-    </row>
-    <row r="40" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z40" s="1"/>
-      <c r="AA40" s="1"/>
-      <c r="AB40" s="1"/>
-    </row>
-    <row r="41" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z41" s="1"/>
-      <c r="AA41" s="1"/>
-      <c r="AB41" s="1"/>
-    </row>
-    <row r="42" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z42" s="1"/>
-      <c r="AA42" s="1"/>
-      <c r="AB42" s="1"/>
-    </row>
-    <row r="43" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z43" s="1"/>
-      <c r="AA43" s="1"/>
-      <c r="AB43" s="1"/>
-    </row>
-    <row r="44" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z44" s="1"/>
-      <c r="AA44" s="1"/>
-      <c r="AB44" s="1"/>
-    </row>
-    <row r="45" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z45" s="1"/>
-      <c r="AA45" s="1"/>
-      <c r="AB45" s="1"/>
-    </row>
-    <row r="46" spans="26:28" x14ac:dyDescent="0.3">
-      <c r="Z46" s="1"/>
-      <c r="AA46" s="1"/>
-      <c r="AB46" s="1"/>
     </row>
     <row r="47" spans="26:28" x14ac:dyDescent="0.3">
       <c r="Z47" s="1"/>
@@ -4254,8 +4173,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A75:A82"/>
-    <mergeCell ref="A84:A91"/>
     <mergeCell ref="A93:A100"/>
     <mergeCell ref="A102:A109"/>
     <mergeCell ref="A21:A28"/>
@@ -4267,6 +4184,8 @@
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="A3:A10"/>
     <mergeCell ref="A12:A19"/>
+    <mergeCell ref="A75:A82"/>
+    <mergeCell ref="A84:A91"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>